<commit_message>
Add daily flying-car, Tesla, Roadster and Musk searches
</commit_message>
<xml_diff>
--- a/data/search_checklist.xlsx
+++ b/data/search_checklist.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索任务" sheetId="1" r:id="R4dc9a913d942472d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="覆盖对象" sheetId="2" r:id="R582fc940a9634bf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="信源索引" sheetId="3" r:id="Rfa185f4d1e954b86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="执行记录模板" sheetId="4" r:id="Rf4912e07bb7a4f92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词库与规则" sheetId="5" r:id="R4ab2218536bc4b5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索任务" sheetId="1" r:id="R211123ec2a524284"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="覆盖对象" sheetId="2" r:id="R1080028266804cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="信源索引" sheetId="3" r:id="Reca69ff2bde24bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="执行记录模板" sheetId="4" r:id="Re81ac1e308ce4f67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="词库与规则" sheetId="5" r:id="Rc07919b8b0174fee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -258,8 +258,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SearchTasks" displayName="SearchTasks" ref="A6:M216" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:M216"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SearchTasks" displayName="SearchTasks" ref="A6:M252" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:M252"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="任务ID"/>
     <x:tableColumn id="2" name="对象ID"/>
@@ -280,8 +280,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CoverageObjects" displayName="CoverageObjects" ref="A6:J180" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:J180"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="CoverageObjects" displayName="CoverageObjects" ref="A6:J213" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:J213"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="对象ID"/>
     <x:tableColumn id="2" name="类别"/>
@@ -326,8 +326,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ExecutionRecords" displayName="ExecutionRecords" ref="A6:N216" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:N216"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ExecutionRecords" displayName="ExecutionRecords" ref="A6:N252" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:N252"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="任务ID"/>
     <x:tableColumn id="2" name="批次ID"/>
@@ -349,8 +349,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="KeywordGroups" displayName="KeywordGroups" ref="A6:E17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:E17"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="KeywordGroups" displayName="KeywordGroups" ref="A6:E19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:E19"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="词组ID"/>
     <x:tableColumn id="2" name="主题"/>
@@ -577,7 +577,7 @@
   <x:sheetData>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>低空新闻联网搜索清单 v1.5</x:v>
+        <x:v>低空新闻联网搜索清单 v1.6</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -594,7 +594,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>共240项任务、204个覆盖对象、117源快照；原230任务及194对象保留，新增6源任务与4企业跟踪任务。</x:v>
+        <x:v>共246项任务、207个覆盖对象、117源快照；保留原240任务/204对象；2026-10-19新增6项飞行汽车独立检索。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -10514,6 +10514,258 @@
       </x:c>
       <x:c r="M246" s="31" t="str">
         <x:v>官方入口与股权关系待核，母集团和低空公司参与身份分别记录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="88" customHeight="1">
+      <x:c r="A247" s="31" t="str">
+        <x:v>FC01-CN</x:v>
+      </x:c>
+      <x:c r="B247" s="31" t="str">
+        <x:v>X-FC01</x:v>
+      </x:c>
+      <x:c r="C247" s="31" t="str">
+        <x:v>跨领域主题</x:v>
+      </x:c>
+      <x:c r="D247" s="31" t="str">
+        <x:v>飞行汽车（中文）</x:v>
+      </x:c>
+      <x:c r="E247" s="31" t="str">
+        <x:v>跨汽车与航空发现</x:v>
+      </x:c>
+      <x:c r="F247" s="31" t="str">
+        <x:v>每日</x:v>
+      </x:c>
+      <x:c r="G247" s="31" t="str">
+        <x:v>增量＋7日回看</x:v>
+      </x:c>
+      <x:c r="H247" s="31" t="str">
+        <x:v>K13</x:v>
+      </x:c>
+      <x:c r="I247" s="31" t="str">
+        <x:v>飞行汽车</x:v>
+      </x:c>
+      <x:c r="J247" s="31" t="str">
+        <x:v>飞行跑车
+陆空两用汽车</x:v>
+      </x:c>
+      <x:c r="K247" s="31" t="str">
+        <x:v>R01;R02;R03</x:v>
+      </x:c>
+      <x:c r="L247" s="31" t="str">
+        <x:v>启用</x:v>
+      </x:c>
+      <x:c r="M247" s="31" t="str">
+        <x:v>每条主式和补充逐行独立执行；命中须追原始发布并逐条登记采用、待核或不采用原因。演示、量产计划、适航及商业运行分开；未读正文不得刊登，不推断ETF或股价影响。新增2026-10-19。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="88" customHeight="1">
+      <x:c r="A248" s="31" t="str">
+        <x:v>FC01-EN</x:v>
+      </x:c>
+      <x:c r="B248" s="31" t="str">
+        <x:v>X-FC01</x:v>
+      </x:c>
+      <x:c r="C248" s="31" t="str">
+        <x:v>跨领域主题</x:v>
+      </x:c>
+      <x:c r="D248" s="31" t="str">
+        <x:v>Flying car（英文）</x:v>
+      </x:c>
+      <x:c r="E248" s="31" t="str">
+        <x:v>跨汽车与航空发现</x:v>
+      </x:c>
+      <x:c r="F248" s="31" t="str">
+        <x:v>每日</x:v>
+      </x:c>
+      <x:c r="G248" s="31" t="str">
+        <x:v>增量＋7日回看</x:v>
+      </x:c>
+      <x:c r="H248" s="31" t="str">
+        <x:v>K13</x:v>
+      </x:c>
+      <x:c r="I248" s="31" t="str">
+        <x:v>"flying car"</x:v>
+      </x:c>
+      <x:c r="J248" s="31" t="str">
+        <x:v>"flying cars"
+"roadable aircraft"</x:v>
+      </x:c>
+      <x:c r="K248" s="31" t="str">
+        <x:v>R01;R02;R03</x:v>
+      </x:c>
+      <x:c r="L248" s="31" t="str">
+        <x:v>启用</x:v>
+      </x:c>
+      <x:c r="M248" s="31" t="str">
+        <x:v>每条主式和补充逐行独立执行；命中须追原始发布并逐条登记采用、待核或不采用原因。演示、量产计划、适航及商业运行分开；未读正文不得刊登，不推断ETF或股价影响。新增2026-10-19。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="88" customHeight="1">
+      <x:c r="A249" s="31" t="str">
+        <x:v>FC02-CN</x:v>
+      </x:c>
+      <x:c r="B249" s="31" t="str">
+        <x:v>E-FC01</x:v>
+      </x:c>
+      <x:c r="C249" s="31" t="str">
+        <x:v>企业</x:v>
+      </x:c>
+      <x:c r="D249" s="31" t="str">
+        <x:v>特斯拉</x:v>
+      </x:c>
+      <x:c r="E249" s="31" t="str">
+        <x:v>企业中文独立检索</x:v>
+      </x:c>
+      <x:c r="F249" s="31" t="str">
+        <x:v>每日</x:v>
+      </x:c>
+      <x:c r="G249" s="31" t="str">
+        <x:v>增量＋7日回看</x:v>
+      </x:c>
+      <x:c r="H249" s="31" t="str">
+        <x:v>K13</x:v>
+      </x:c>
+      <x:c r="I249" s="31" t="str">
+        <x:v>特斯拉 飞行</x:v>
+      </x:c>
+      <x:c r="J249" s="31" t="str">
+        <x:v>特斯拉 飞行汽车
+特斯拉 Roadster</x:v>
+      </x:c>
+      <x:c r="K249" s="31" t="str">
+        <x:v>R01;R02;R03;O09</x:v>
+      </x:c>
+      <x:c r="L249" s="31" t="str">
+        <x:v>启用</x:v>
+      </x:c>
+      <x:c r="M249" s="31" t="str">
+        <x:v>每条主式和补充逐行独立执行；命中须追原始发布并逐条登记采用、待核或不采用原因。演示、量产计划、适航及商业运行分开；未读正文不得刊登，不推断ETF或股价影响。新增2026-10-19。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="88" customHeight="1">
+      <x:c r="A250" s="31" t="str">
+        <x:v>FC02-EN</x:v>
+      </x:c>
+      <x:c r="B250" s="31" t="str">
+        <x:v>E-FC01</x:v>
+      </x:c>
+      <x:c r="C250" s="31" t="str">
+        <x:v>企业</x:v>
+      </x:c>
+      <x:c r="D250" s="31" t="str">
+        <x:v>Tesla</x:v>
+      </x:c>
+      <x:c r="E250" s="31" t="str">
+        <x:v>企业英文独立检索</x:v>
+      </x:c>
+      <x:c r="F250" s="31" t="str">
+        <x:v>每日</x:v>
+      </x:c>
+      <x:c r="G250" s="31" t="str">
+        <x:v>增量＋7日回看</x:v>
+      </x:c>
+      <x:c r="H250" s="31" t="str">
+        <x:v>K13</x:v>
+      </x:c>
+      <x:c r="I250" s="31" t="str">
+        <x:v>Tesla flying</x:v>
+      </x:c>
+      <x:c r="J250" s="31" t="str">
+        <x:v>Tesla "flying car"
+Tesla Roadster</x:v>
+      </x:c>
+      <x:c r="K250" s="31" t="str">
+        <x:v>R01;R02;R03;O09</x:v>
+      </x:c>
+      <x:c r="L250" s="31" t="str">
+        <x:v>启用</x:v>
+      </x:c>
+      <x:c r="M250" s="31" t="str">
+        <x:v>每条主式和补充逐行独立执行；命中须追原始发布并逐条登记采用、待核或不采用原因。演示、量产计划、适航及商业运行分开；未读正文不得刊登，不推断ETF或股价影响。新增2026-10-19。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="88" customHeight="1">
+      <x:c r="A251" s="31" t="str">
+        <x:v>FC03</x:v>
+      </x:c>
+      <x:c r="B251" s="31" t="str">
+        <x:v>P-FC01</x:v>
+      </x:c>
+      <x:c r="C251" s="31" t="str">
+        <x:v>产品</x:v>
+      </x:c>
+      <x:c r="D251" s="31" t="str">
+        <x:v>Tesla Roadster</x:v>
+      </x:c>
+      <x:c r="E251" s="31" t="str">
+        <x:v>产品名称独立检索</x:v>
+      </x:c>
+      <x:c r="F251" s="31" t="str">
+        <x:v>每日</x:v>
+      </x:c>
+      <x:c r="G251" s="31" t="str">
+        <x:v>增量＋7日回看</x:v>
+      </x:c>
+      <x:c r="H251" s="31" t="str">
+        <x:v>K13</x:v>
+      </x:c>
+      <x:c r="I251" s="31" t="str">
+        <x:v>Roadster</x:v>
+      </x:c>
+      <x:c r="J251" s="31" t="str">
+        <x:v>Roadster thrusters
+Roadster flight</x:v>
+      </x:c>
+      <x:c r="K251" s="31" t="str">
+        <x:v>R01;R02;R03;O09</x:v>
+      </x:c>
+      <x:c r="L251" s="31" t="str">
+        <x:v>启用</x:v>
+      </x:c>
+      <x:c r="M251" s="31" t="str">
+        <x:v>每条主式和补充逐行独立执行；命中须追原始发布并逐条登记采用、待核或不采用原因。演示、量产计划、适航及商业运行分开；未读正文不得刊登，不推断ETF或股价影响。新增2026-10-19。筛除服饰品牌及无关车型；2017概念与本次进展分开。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="88" customHeight="1">
+      <x:c r="A252" s="31" t="str">
+        <x:v>FC04</x:v>
+      </x:c>
+      <x:c r="B252" s="31" t="str">
+        <x:v>E-FC01</x:v>
+      </x:c>
+      <x:c r="C252" s="31" t="str">
+        <x:v>企业发言</x:v>
+      </x:c>
+      <x:c r="D252" s="31" t="str">
+        <x:v>马斯克相关飞行产品声明</x:v>
+      </x:c>
+      <x:c r="E252" s="31" t="str">
+        <x:v>人物与别名独立检索</x:v>
+      </x:c>
+      <x:c r="F252" s="31" t="str">
+        <x:v>每日</x:v>
+      </x:c>
+      <x:c r="G252" s="31" t="str">
+        <x:v>增量＋7日回看</x:v>
+      </x:c>
+      <x:c r="H252" s="31" t="str">
+        <x:v>K13</x:v>
+      </x:c>
+      <x:c r="I252" s="31" t="str">
+        <x:v>马斯克 飞行汽车</x:v>
+      </x:c>
+      <x:c r="J252" s="31" t="str">
+        <x:v>"Elon Musk" "flying car"
+马斯克 Roadster</x:v>
+      </x:c>
+      <x:c r="K252" s="31" t="str">
+        <x:v>R01;R02;R03;O09</x:v>
+      </x:c>
+      <x:c r="L252" s="31" t="str">
+        <x:v>启用</x:v>
+      </x:c>
+      <x:c r="M252" s="31" t="str">
+        <x:v>每条主式和补充逐行独立执行；命中须追原始发布并逐条登记采用、待核或不采用原因。演示、量产计划、适航及商业运行分开；未读正文不得刊登，不推断ETF或股价影响。新增2026-10-19。核发言主体及所指企业；SpaceX、Tesla、第三方公司分开。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10532,7 +10784,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a28f54765784e12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ada46df93384a42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10569,7 +10821,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>共204个覆盖对象；新增候选源6个及企业4家；企业官网未核不编造地址。</x:v>
+        <x:v>207个覆盖对象；新增跨领域飞行汽车、Tesla与Roadster三个对象，原204对象及ID保留。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -17043,6 +17295,102 @@
         <x:v>仅记录协办，不当主办；不推定与地空产融同集团</x:v>
       </x:c>
     </x:row>
+    <x:row r="211" ht="92" customHeight="1">
+      <x:c r="A211" s="31" t="str">
+        <x:v>X-FC01</x:v>
+      </x:c>
+      <x:c r="B211" s="31" t="str">
+        <x:v>跨领域主题</x:v>
+      </x:c>
+      <x:c r="C211" s="31" t="str">
+        <x:v>飞行汽车与陆空两用产品</x:v>
+      </x:c>
+      <x:c r="D211" s="31" t="str">
+        <x:v>全国及海外</x:v>
+      </x:c>
+      <x:c r="E211" s="31" t="str">
+        <x:v>产品展示、研发、监管与应用</x:v>
+      </x:c>
+      <x:c r="F211" s="31" t="str">
+        <x:v>每日</x:v>
+      </x:c>
+      <x:c r="G211" s="31" t="str">
+        <x:v>R01;R02;R03</x:v>
+      </x:c>
+      <x:c r="H211" s="31" t="str">
+        <x:v>主题覆盖；不是稳定采集来源</x:v>
+      </x:c>
+      <x:c r="I211" s="31" t="str">
+        <x:v>2026-10-19：针对Roadster线索遗漏新增</x:v>
+      </x:c>
+      <x:c r="J211" s="31" t="str">
+        <x:v>中文与英文分别查，兼顾清单外企业；不能因标题未含eVTOL而排除</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="92" customHeight="1">
+      <x:c r="A212" s="31" t="str">
+        <x:v>E-FC01</x:v>
+      </x:c>
+      <x:c r="B212" s="31" t="str">
+        <x:v>企业</x:v>
+      </x:c>
+      <x:c r="C212" s="31" t="str">
+        <x:v>Tesla, Inc.（特斯拉）</x:v>
+      </x:c>
+      <x:c r="D212" s="31" t="str">
+        <x:v>美国及相关海外市场</x:v>
+      </x:c>
+      <x:c r="E212" s="31" t="str">
+        <x:v>Roadster与飞行相关企业发布及管理层声明</x:v>
+      </x:c>
+      <x:c r="F212" s="31" t="str">
+        <x:v>每日</x:v>
+      </x:c>
+      <x:c r="G212" s="31" t="str">
+        <x:v>R01;R02;R03;O09</x:v>
+      </x:c>
+      <x:c r="H212" s="31" t="str">
+        <x:v>官网管理层页已读；产品页只读到脚注，全文与连续采集未验收</x:v>
+      </x:c>
+      <x:c r="I212" s="31" t="str">
+        <x:v>2026-10-19；https://www.tesla.com/elon-musk；https://www.tesla.com/roadster</x:v>
+      </x:c>
+      <x:c r="J212" s="31" t="str">
+        <x:v>仅跟踪飞行相关消息；马斯克发言保留归属，Tesla与SpaceX分开；官网尚未登记为稳定信源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="92" customHeight="1">
+      <x:c r="A213" s="31" t="str">
+        <x:v>P-FC01</x:v>
+      </x:c>
+      <x:c r="B213" s="31" t="str">
+        <x:v>产品</x:v>
+      </x:c>
+      <x:c r="C213" s="31" t="str">
+        <x:v>Tesla Roadster（飞行相关版本）</x:v>
+      </x:c>
+      <x:c r="D213" s="31" t="str">
+        <x:v>美国及相关市场</x:v>
+      </x:c>
+      <x:c r="E213" s="31" t="str">
+        <x:v>演示、预订、量产、认证与交付</x:v>
+      </x:c>
+      <x:c r="F213" s="31" t="str">
+        <x:v>每日</x:v>
+      </x:c>
+      <x:c r="G213" s="31" t="str">
+        <x:v>R01;R02;R03;O09</x:v>
+      </x:c>
+      <x:c r="H213" s="31" t="str">
+        <x:v>Tesla官方产品入口已定位；可读内容有限，发布会原始视频待核</x:v>
+      </x:c>
+      <x:c r="I213" s="31" t="str">
+        <x:v>2026-10-19；https://www.tesla.com/roadster</x:v>
+      </x:c>
+      <x:c r="J213" s="31" t="str">
+        <x:v>Roadster单独检索后筛相关性；区分Performance、Thrust、Rocket版本，预订不当交付，短时腾空不写商业载客</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="H7:H166">
     <x:cfRule type="expression" dxfId="1" priority="1">
@@ -17051,7 +17399,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4de226398f4346fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cfc205c888e4b82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23523,7 +23871,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1db384724a864cab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84390dd5c20b4da7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23568,7 +23916,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>240行空模板；实际执行另存日期/批次文件，未执行不倒填。</x:v>
+        <x:v>246行空模板；实际执行另存日期/批次文件，未执行不倒填。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -29135,6 +29483,138 @@
       <x:c r="L246" s="31"/>
       <x:c r="M246" s="31"/>
       <x:c r="N246" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247">
+      <x:c r="A247" s="31" t="str">
+        <x:v>FC01-CN</x:v>
+      </x:c>
+      <x:c r="B247" s="31"/>
+      <x:c r="C247" s="31"/>
+      <x:c r="D247" s="31"/>
+      <x:c r="E247" s="31"/>
+      <x:c r="F247" s="31"/>
+      <x:c r="G247" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H247" s="31"/>
+      <x:c r="I247" s="31"/>
+      <x:c r="J247" s="31"/>
+      <x:c r="K247" s="31"/>
+      <x:c r="L247" s="31"/>
+      <x:c r="M247" s="31"/>
+      <x:c r="N247" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248">
+      <x:c r="A248" s="31" t="str">
+        <x:v>FC01-EN</x:v>
+      </x:c>
+      <x:c r="B248" s="31"/>
+      <x:c r="C248" s="31"/>
+      <x:c r="D248" s="31"/>
+      <x:c r="E248" s="31"/>
+      <x:c r="F248" s="31"/>
+      <x:c r="G248" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H248" s="31"/>
+      <x:c r="I248" s="31"/>
+      <x:c r="J248" s="31"/>
+      <x:c r="K248" s="31"/>
+      <x:c r="L248" s="31"/>
+      <x:c r="M248" s="31"/>
+      <x:c r="N248" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249">
+      <x:c r="A249" s="31" t="str">
+        <x:v>FC02-CN</x:v>
+      </x:c>
+      <x:c r="B249" s="31"/>
+      <x:c r="C249" s="31"/>
+      <x:c r="D249" s="31"/>
+      <x:c r="E249" s="31"/>
+      <x:c r="F249" s="31"/>
+      <x:c r="G249" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H249" s="31"/>
+      <x:c r="I249" s="31"/>
+      <x:c r="J249" s="31"/>
+      <x:c r="K249" s="31"/>
+      <x:c r="L249" s="31"/>
+      <x:c r="M249" s="31"/>
+      <x:c r="N249" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250">
+      <x:c r="A250" s="31" t="str">
+        <x:v>FC02-EN</x:v>
+      </x:c>
+      <x:c r="B250" s="31"/>
+      <x:c r="C250" s="31"/>
+      <x:c r="D250" s="31"/>
+      <x:c r="E250" s="31"/>
+      <x:c r="F250" s="31"/>
+      <x:c r="G250" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H250" s="31"/>
+      <x:c r="I250" s="31"/>
+      <x:c r="J250" s="31"/>
+      <x:c r="K250" s="31"/>
+      <x:c r="L250" s="31"/>
+      <x:c r="M250" s="31"/>
+      <x:c r="N250" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251">
+      <x:c r="A251" s="31" t="str">
+        <x:v>FC03</x:v>
+      </x:c>
+      <x:c r="B251" s="31"/>
+      <x:c r="C251" s="31"/>
+      <x:c r="D251" s="31"/>
+      <x:c r="E251" s="31"/>
+      <x:c r="F251" s="31"/>
+      <x:c r="G251" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H251" s="31"/>
+      <x:c r="I251" s="31"/>
+      <x:c r="J251" s="31"/>
+      <x:c r="K251" s="31"/>
+      <x:c r="L251" s="31"/>
+      <x:c r="M251" s="31"/>
+      <x:c r="N251" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252">
+      <x:c r="A252" s="31" t="str">
+        <x:v>FC04</x:v>
+      </x:c>
+      <x:c r="B252" s="31"/>
+      <x:c r="C252" s="31"/>
+      <x:c r="D252" s="31"/>
+      <x:c r="E252" s="31"/>
+      <x:c r="F252" s="31"/>
+      <x:c r="G252" s="31" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H252" s="31"/>
+      <x:c r="I252" s="31"/>
+      <x:c r="J252" s="31"/>
+      <x:c r="K252" s="31"/>
+      <x:c r="L252" s="31"/>
+      <x:c r="M252" s="31"/>
+      <x:c r="N252" s="31" t="str">
         <x:v>未执行</x:v>
       </x:c>
     </x:row>
@@ -29156,7 +29636,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a12d7d78fe84c55"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R034f21540f7d4919"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29183,7 +29663,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>词库版本1.1，2026-10-18新增K06人才与赛事；其余原词组及执行规则保留，时间统一为北京时间。</x:v>
+        <x:v>词库版本1.2；保留原词组与规则，2026-10-19新增K13飞行汽车与跨领域产品独立检索。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -29427,6 +29907,23 @@
         <x:v>主办/承办/集团支持身份分开；报名截止与报到时间分开，报名入口异常另记</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" ht="56" customHeight="1">
+      <x:c r="A19" s="32" t="str">
+        <x:v>K13</x:v>
+      </x:c>
+      <x:c r="B19" s="32" t="str">
+        <x:v>飞行汽车与跨领域产品</x:v>
+      </x:c>
+      <x:c r="C19" s="32" t="str">
+        <x:v>飞行汽车；飞行跑车；陆空两用汽车；flying car；roadable aircraft；Tesla；Roadster；马斯克；Elon Musk</x:v>
+      </x:c>
+      <x:c r="D19" s="32" t="str">
+        <x:v>发布；演示；thrusters；flight；预订；量产；认证；交付</x:v>
+      </x:c>
+      <x:c r="E19" s="32" t="str">
+        <x:v>同义词及主体分条查询；命中逐条登记去向；展示、承诺、认证与交付分开</x:v>
+      </x:c>
+    </x:row>
     <x:row r="21" ht="28" customHeight="1">
       <x:c r="A21" s="28" t="str">
         <x:v>序号</x:v>
@@ -29668,7 +30165,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9e5385e5363476a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R753c23bc15d44c8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>